<commit_message>
feat: update 'INFO OBRAS' file
</commit_message>
<xml_diff>
--- a/obras-arquivos/INFO OBRAS.xlsx
+++ b/obras-arquivos/INFO OBRAS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dougl\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dougl\Desktop\Eng\Work\RELATÓRIOS\prefeitura-docs\obras-arquivos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49CCFC77-130D-410C-A581-7B5227FB7DD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D918EB44-CEC1-4865-BC60-B474020E1BE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{72B2B929-4AC3-4F94-90DA-D90B6998E1FC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{72B2B929-4AC3-4F94-90DA-D90B6998E1FC}"/>
   </bookViews>
   <sheets>
     <sheet name="ESCOLA 6 SALAS (PRIMEIRA ETAPA)" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="101">
   <si>
     <t>DADOS GERAIS</t>
   </si>
@@ -301,9 +301,6 @@
   </si>
   <si>
     <t>VALOR ACUMULADO</t>
-  </si>
-  <si>
-    <t>Rescindido</t>
   </si>
   <si>
     <t>O valor total passará de R$ 1.039.467,57 para R$ 1.249.356,45</t>
@@ -434,7 +431,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -471,12 +468,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="52">
     <border>
@@ -1134,7 +1125,7 @@
     <xf numFmtId="44" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="203">
+  <cellXfs count="201">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1249,37 +1240,367 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1294,10 +1615,22 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1315,382 +1648,52 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1699,37 +1702,19 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2110,27 +2095,27 @@
     </row>
     <row r="2" spans="1:38" ht="21" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
-      <c r="B2" s="99" t="s">
+      <c r="B2" s="105" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="100"/>
-      <c r="D2" s="100"/>
-      <c r="E2" s="100"/>
-      <c r="F2" s="100"/>
-      <c r="G2" s="100"/>
-      <c r="H2" s="100"/>
-      <c r="I2" s="100"/>
-      <c r="J2" s="100"/>
-      <c r="K2" s="100"/>
-      <c r="L2" s="100"/>
-      <c r="M2" s="100"/>
-      <c r="N2" s="100"/>
-      <c r="O2" s="100"/>
-      <c r="P2" s="100"/>
-      <c r="Q2" s="100"/>
-      <c r="R2" s="100"/>
-      <c r="S2" s="100"/>
-      <c r="T2" s="101"/>
+      <c r="C2" s="106"/>
+      <c r="D2" s="106"/>
+      <c r="E2" s="106"/>
+      <c r="F2" s="106"/>
+      <c r="G2" s="106"/>
+      <c r="H2" s="106"/>
+      <c r="I2" s="106"/>
+      <c r="J2" s="106"/>
+      <c r="K2" s="106"/>
+      <c r="L2" s="106"/>
+      <c r="M2" s="106"/>
+      <c r="N2" s="106"/>
+      <c r="O2" s="106"/>
+      <c r="P2" s="106"/>
+      <c r="Q2" s="106"/>
+      <c r="R2" s="106"/>
+      <c r="S2" s="106"/>
+      <c r="T2" s="107"/>
       <c r="U2" s="4"/>
       <c r="V2" s="4"/>
       <c r="W2" s="4"/>
@@ -2152,27 +2137,27 @@
     </row>
     <row r="3" spans="1:38" ht="40.799999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2"/>
-      <c r="B3" s="110" t="s">
+      <c r="B3" s="118" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="111"/>
-      <c r="D3" s="111"/>
-      <c r="E3" s="111"/>
-      <c r="F3" s="111"/>
-      <c r="G3" s="112"/>
-      <c r="H3" s="112"/>
-      <c r="I3" s="112"/>
-      <c r="J3" s="112"/>
-      <c r="K3" s="112"/>
-      <c r="L3" s="112"/>
-      <c r="M3" s="112"/>
-      <c r="N3" s="112"/>
-      <c r="O3" s="112"/>
-      <c r="P3" s="112"/>
-      <c r="Q3" s="112"/>
-      <c r="R3" s="112"/>
-      <c r="S3" s="112"/>
-      <c r="T3" s="113"/>
+      <c r="C3" s="119"/>
+      <c r="D3" s="119"/>
+      <c r="E3" s="119"/>
+      <c r="F3" s="119"/>
+      <c r="G3" s="120"/>
+      <c r="H3" s="120"/>
+      <c r="I3" s="120"/>
+      <c r="J3" s="120"/>
+      <c r="K3" s="120"/>
+      <c r="L3" s="120"/>
+      <c r="M3" s="120"/>
+      <c r="N3" s="120"/>
+      <c r="O3" s="120"/>
+      <c r="P3" s="120"/>
+      <c r="Q3" s="120"/>
+      <c r="R3" s="120"/>
+      <c r="S3" s="120"/>
+      <c r="T3" s="121"/>
       <c r="U3" s="4"/>
       <c r="V3" s="4"/>
       <c r="W3" s="4"/>
@@ -2234,29 +2219,29 @@
     </row>
     <row r="5" spans="1:38" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4"/>
-      <c r="B5" s="106" t="s">
+      <c r="B5" s="114" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="107"/>
-      <c r="D5" s="107"/>
-      <c r="E5" s="107"/>
-      <c r="F5" s="107"/>
-      <c r="G5" s="107"/>
-      <c r="H5" s="107"/>
-      <c r="I5" s="107"/>
-      <c r="J5" s="108"/>
-      <c r="K5" s="109"/>
+      <c r="C5" s="115"/>
+      <c r="D5" s="115"/>
+      <c r="E5" s="115"/>
+      <c r="F5" s="115"/>
+      <c r="G5" s="115"/>
+      <c r="H5" s="115"/>
+      <c r="I5" s="115"/>
+      <c r="J5" s="116"/>
+      <c r="K5" s="117"/>
       <c r="L5" s="19"/>
-      <c r="M5" s="103" t="s">
+      <c r="M5" s="111" t="s">
         <v>27</v>
       </c>
-      <c r="N5" s="104"/>
-      <c r="O5" s="104"/>
-      <c r="P5" s="104"/>
-      <c r="Q5" s="104"/>
-      <c r="R5" s="104"/>
-      <c r="S5" s="104"/>
-      <c r="T5" s="105"/>
+      <c r="N5" s="112"/>
+      <c r="O5" s="112"/>
+      <c r="P5" s="112"/>
+      <c r="Q5" s="112"/>
+      <c r="R5" s="112"/>
+      <c r="S5" s="112"/>
+      <c r="T5" s="113"/>
       <c r="U5" s="4"/>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -2278,37 +2263,37 @@
     </row>
     <row r="6" spans="1:38" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="18"/>
-      <c r="B6" s="77" t="s">
+      <c r="B6" s="133" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="78"/>
-      <c r="D6" s="78"/>
-      <c r="E6" s="79"/>
-      <c r="F6" s="79"/>
-      <c r="G6" s="77" t="s">
+      <c r="C6" s="134"/>
+      <c r="D6" s="134"/>
+      <c r="E6" s="135"/>
+      <c r="F6" s="135"/>
+      <c r="G6" s="133" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="78"/>
-      <c r="I6" s="78"/>
-      <c r="J6" s="79"/>
-      <c r="K6" s="128"/>
+      <c r="H6" s="134"/>
+      <c r="I6" s="134"/>
+      <c r="J6" s="135"/>
+      <c r="K6" s="136"/>
       <c r="L6" s="20"/>
-      <c r="M6" s="51" t="s">
+      <c r="M6" s="93" t="s">
         <v>39</v>
       </c>
-      <c r="N6" s="52"/>
-      <c r="O6" s="44" t="s">
+      <c r="N6" s="94"/>
+      <c r="O6" s="169" t="s">
         <v>59</v>
       </c>
-      <c r="P6" s="44"/>
-      <c r="Q6" s="57" t="s">
+      <c r="P6" s="169"/>
+      <c r="Q6" s="161" t="s">
         <v>37</v>
       </c>
-      <c r="R6" s="57"/>
-      <c r="S6" s="53">
+      <c r="R6" s="161"/>
+      <c r="S6" s="163">
         <v>1252370.6000000001</v>
       </c>
-      <c r="T6" s="54"/>
+      <c r="T6" s="164"/>
       <c r="U6" s="18"/>
       <c r="V6" s="18"/>
       <c r="W6" s="18"/>
@@ -2330,33 +2315,33 @@
     </row>
     <row r="7" spans="1:38" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="18"/>
-      <c r="B7" s="80"/>
-      <c r="C7" s="81"/>
-      <c r="D7" s="81"/>
-      <c r="E7" s="82"/>
-      <c r="F7" s="82"/>
-      <c r="G7" s="80"/>
-      <c r="H7" s="81"/>
-      <c r="I7" s="81"/>
-      <c r="J7" s="82"/>
-      <c r="K7" s="129"/>
+      <c r="B7" s="137"/>
+      <c r="C7" s="138"/>
+      <c r="D7" s="138"/>
+      <c r="E7" s="139"/>
+      <c r="F7" s="139"/>
+      <c r="G7" s="137"/>
+      <c r="H7" s="138"/>
+      <c r="I7" s="138"/>
+      <c r="J7" s="139"/>
+      <c r="K7" s="140"/>
       <c r="L7" s="20"/>
-      <c r="M7" s="51" t="s">
+      <c r="M7" s="93" t="s">
         <v>32</v>
       </c>
-      <c r="N7" s="76"/>
-      <c r="O7" s="45" t="s">
-        <v>87</v>
-      </c>
-      <c r="P7" s="46"/>
-      <c r="Q7" s="58" t="s">
+      <c r="N7" s="160"/>
+      <c r="O7" s="199" t="s">
+        <v>60</v>
+      </c>
+      <c r="P7" s="200"/>
+      <c r="Q7" s="162" t="s">
         <v>55</v>
       </c>
-      <c r="R7" s="52"/>
-      <c r="S7" s="53" t="s">
+      <c r="R7" s="94"/>
+      <c r="S7" s="163" t="s">
         <v>65</v>
       </c>
-      <c r="T7" s="54"/>
+      <c r="T7" s="164"/>
       <c r="U7" s="18"/>
       <c r="V7" s="18"/>
       <c r="W7" s="18"/>
@@ -2378,41 +2363,41 @@
     </row>
     <row r="8" spans="1:38" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
-      <c r="B8" s="69" t="s">
+      <c r="B8" s="82" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="130"/>
-      <c r="D8" s="118" t="s">
+      <c r="C8" s="83"/>
+      <c r="D8" s="97" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="119"/>
-      <c r="F8" s="119"/>
-      <c r="G8" s="69" t="s">
+      <c r="E8" s="98"/>
+      <c r="F8" s="98"/>
+      <c r="G8" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="H8" s="130"/>
-      <c r="I8" s="86" t="s">
+      <c r="H8" s="83"/>
+      <c r="I8" s="141" t="s">
         <v>22</v>
       </c>
-      <c r="J8" s="87"/>
-      <c r="K8" s="88"/>
+      <c r="J8" s="142"/>
+      <c r="K8" s="143"/>
       <c r="L8" s="19"/>
-      <c r="M8" s="51" t="s">
+      <c r="M8" s="93" t="s">
         <v>33</v>
       </c>
-      <c r="N8" s="52"/>
-      <c r="O8" s="47" t="s">
+      <c r="N8" s="94"/>
+      <c r="O8" s="170" t="s">
         <v>61</v>
       </c>
-      <c r="P8" s="47"/>
-      <c r="Q8" s="52" t="s">
+      <c r="P8" s="170"/>
+      <c r="Q8" s="94" t="s">
         <v>56</v>
       </c>
-      <c r="R8" s="52"/>
-      <c r="S8" s="55">
+      <c r="R8" s="94"/>
+      <c r="S8" s="165">
         <v>44517</v>
       </c>
-      <c r="T8" s="56"/>
+      <c r="T8" s="166"/>
       <c r="U8" s="4"/>
       <c r="V8" s="4"/>
       <c r="W8" s="4"/>
@@ -2434,41 +2419,41 @@
     </row>
     <row r="9" spans="1:38" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
-      <c r="B9" s="71" t="s">
+      <c r="B9" s="84" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="83"/>
-      <c r="D9" s="50" t="s">
+      <c r="C9" s="85"/>
+      <c r="D9" s="99" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="120"/>
-      <c r="F9" s="120"/>
-      <c r="G9" s="71" t="s">
+      <c r="E9" s="100"/>
+      <c r="F9" s="100"/>
+      <c r="G9" s="84" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="83"/>
-      <c r="I9" s="89">
+      <c r="H9" s="85"/>
+      <c r="I9" s="144">
         <v>45027</v>
       </c>
-      <c r="J9" s="90"/>
-      <c r="K9" s="91"/>
+      <c r="J9" s="145"/>
+      <c r="K9" s="146"/>
       <c r="L9" s="19"/>
-      <c r="M9" s="51" t="s">
+      <c r="M9" s="93" t="s">
         <v>34</v>
       </c>
-      <c r="N9" s="52"/>
-      <c r="O9" s="48" t="s">
+      <c r="N9" s="94"/>
+      <c r="O9" s="171" t="s">
         <v>62</v>
       </c>
-      <c r="P9" s="48"/>
-      <c r="Q9" s="52" t="s">
+      <c r="P9" s="171"/>
+      <c r="Q9" s="94" t="s">
         <v>15</v>
       </c>
-      <c r="R9" s="52"/>
-      <c r="S9" s="55">
+      <c r="R9" s="94"/>
+      <c r="S9" s="165">
         <v>44511</v>
       </c>
-      <c r="T9" s="56"/>
+      <c r="T9" s="166"/>
       <c r="U9" s="4"/>
       <c r="V9" s="4"/>
       <c r="W9" s="4"/>
@@ -2490,41 +2475,41 @@
     </row>
     <row r="10" spans="1:38" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
-      <c r="B10" s="71" t="s">
+      <c r="B10" s="84" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="83"/>
-      <c r="D10" s="121">
+      <c r="C10" s="85"/>
+      <c r="D10" s="126">
         <v>44980</v>
       </c>
-      <c r="E10" s="122"/>
-      <c r="F10" s="122"/>
-      <c r="G10" s="71" t="s">
+      <c r="E10" s="127"/>
+      <c r="F10" s="127"/>
+      <c r="G10" s="84" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="83"/>
-      <c r="I10" s="92">
+      <c r="H10" s="85"/>
+      <c r="I10" s="147">
         <v>1039467.57</v>
       </c>
-      <c r="J10" s="93"/>
-      <c r="K10" s="94"/>
+      <c r="J10" s="148"/>
+      <c r="K10" s="149"/>
       <c r="L10" s="19"/>
-      <c r="M10" s="51" t="s">
+      <c r="M10" s="93" t="s">
         <v>35</v>
       </c>
-      <c r="N10" s="52"/>
-      <c r="O10" s="48" t="s">
+      <c r="N10" s="94"/>
+      <c r="O10" s="171" t="s">
         <v>63</v>
       </c>
-      <c r="P10" s="48"/>
-      <c r="Q10" s="52" t="s">
+      <c r="P10" s="171"/>
+      <c r="Q10" s="94" t="s">
         <v>16</v>
       </c>
-      <c r="R10" s="52"/>
-      <c r="S10" s="55">
+      <c r="R10" s="94"/>
+      <c r="S10" s="165">
         <v>44895</v>
       </c>
-      <c r="T10" s="56"/>
+      <c r="T10" s="166"/>
       <c r="U10" s="4"/>
       <c r="V10" s="4"/>
       <c r="W10" s="4"/>
@@ -2546,41 +2531,41 @@
     </row>
     <row r="11" spans="1:38" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4"/>
-      <c r="B11" s="71" t="s">
+      <c r="B11" s="84" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="83"/>
-      <c r="D11" s="123">
+      <c r="C11" s="85"/>
+      <c r="D11" s="128">
         <v>1039467.57</v>
       </c>
-      <c r="E11" s="124"/>
-      <c r="F11" s="124"/>
-      <c r="G11" s="71" t="s">
+      <c r="E11" s="129"/>
+      <c r="F11" s="129"/>
+      <c r="G11" s="84" t="s">
         <v>15</v>
       </c>
-      <c r="H11" s="83"/>
-      <c r="I11" s="89">
+      <c r="H11" s="85"/>
+      <c r="I11" s="144">
         <v>45027</v>
       </c>
-      <c r="J11" s="90"/>
-      <c r="K11" s="91"/>
+      <c r="J11" s="145"/>
+      <c r="K11" s="146"/>
       <c r="L11" s="19"/>
-      <c r="M11" s="98" t="s">
+      <c r="M11" s="95" t="s">
         <v>36</v>
       </c>
-      <c r="N11" s="75"/>
-      <c r="O11" s="49" t="s">
+      <c r="N11" s="96"/>
+      <c r="O11" s="172" t="s">
         <v>64</v>
       </c>
-      <c r="P11" s="49"/>
-      <c r="Q11" s="75" t="s">
+      <c r="P11" s="172"/>
+      <c r="Q11" s="96" t="s">
         <v>57</v>
       </c>
-      <c r="R11" s="75"/>
-      <c r="S11" s="73">
+      <c r="R11" s="96"/>
+      <c r="S11" s="158">
         <v>0</v>
       </c>
-      <c r="T11" s="74"/>
+      <c r="T11" s="159"/>
       <c r="U11" s="4"/>
       <c r="V11" s="4"/>
       <c r="W11" s="4"/>
@@ -2602,24 +2587,24 @@
     </row>
     <row r="12" spans="1:38" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4"/>
-      <c r="B12" s="71" t="s">
+      <c r="B12" s="84" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="83"/>
-      <c r="D12" s="123">
+      <c r="C12" s="85"/>
+      <c r="D12" s="128">
         <v>1252370</v>
       </c>
-      <c r="E12" s="124"/>
-      <c r="F12" s="124"/>
-      <c r="G12" s="84" t="s">
+      <c r="E12" s="129"/>
+      <c r="F12" s="129"/>
+      <c r="G12" s="86" t="s">
         <v>16</v>
       </c>
-      <c r="H12" s="85"/>
-      <c r="I12" s="95">
+      <c r="H12" s="87"/>
+      <c r="I12" s="150">
         <v>45291</v>
       </c>
-      <c r="J12" s="96"/>
-      <c r="K12" s="97"/>
+      <c r="J12" s="151"/>
+      <c r="K12" s="152"/>
       <c r="L12" s="19"/>
       <c r="M12" s="8" t="s">
         <v>38</v>
@@ -2652,33 +2637,33 @@
     </row>
     <row r="13" spans="1:38" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4"/>
-      <c r="B13" s="114" t="s">
+      <c r="B13" s="122" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="115"/>
-      <c r="D13" s="125" t="s">
+      <c r="C13" s="123"/>
+      <c r="D13" s="130" t="s">
         <v>58</v>
       </c>
-      <c r="E13" s="126"/>
-      <c r="F13" s="126"/>
-      <c r="G13" s="64" t="s">
+      <c r="E13" s="131"/>
+      <c r="F13" s="131"/>
+      <c r="G13" s="108" t="s">
         <v>17</v>
       </c>
-      <c r="H13" s="65"/>
-      <c r="I13" s="66"/>
-      <c r="J13" s="67"/>
-      <c r="K13" s="68"/>
+      <c r="H13" s="109"/>
+      <c r="I13" s="153"/>
+      <c r="J13" s="154"/>
+      <c r="K13" s="155"/>
       <c r="L13" s="30"/>
-      <c r="M13" s="61" t="s">
+      <c r="M13" s="175" t="s">
         <v>38</v>
       </c>
-      <c r="N13" s="62"/>
-      <c r="O13" s="62"/>
-      <c r="P13" s="62"/>
-      <c r="Q13" s="62"/>
-      <c r="R13" s="62"/>
-      <c r="S13" s="62"/>
-      <c r="T13" s="63"/>
+      <c r="N13" s="176"/>
+      <c r="O13" s="176"/>
+      <c r="P13" s="176"/>
+      <c r="Q13" s="176"/>
+      <c r="R13" s="176"/>
+      <c r="S13" s="176"/>
+      <c r="T13" s="177"/>
       <c r="U13" s="4"/>
       <c r="V13" s="4"/>
       <c r="W13" s="4"/>
@@ -2700,19 +2685,19 @@
     </row>
     <row r="14" spans="1:38" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
-      <c r="B14" s="114"/>
-      <c r="C14" s="115"/>
-      <c r="D14" s="125"/>
-      <c r="E14" s="126"/>
-      <c r="F14" s="126"/>
-      <c r="G14" s="69" t="s">
+      <c r="B14" s="122"/>
+      <c r="C14" s="123"/>
+      <c r="D14" s="130"/>
+      <c r="E14" s="131"/>
+      <c r="F14" s="131"/>
+      <c r="G14" s="82" t="s">
         <v>18</v>
       </c>
-      <c r="H14" s="70"/>
-      <c r="I14" s="157" t="s">
-        <v>89</v>
-      </c>
-      <c r="J14" s="158"/>
+      <c r="H14" s="156"/>
+      <c r="I14" s="62" t="s">
+        <v>88</v>
+      </c>
+      <c r="J14" s="63"/>
       <c r="K14" s="32">
         <v>209888.88</v>
       </c>
@@ -2720,10 +2705,10 @@
       <c r="M14" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="N14" s="59" t="s">
+      <c r="N14" s="173" t="s">
         <v>41</v>
       </c>
-      <c r="O14" s="60"/>
+      <c r="O14" s="174"/>
       <c r="P14" s="7" t="s">
         <v>42</v>
       </c>
@@ -2760,26 +2745,26 @@
     </row>
     <row r="15" spans="1:38" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4"/>
-      <c r="B15" s="114"/>
-      <c r="C15" s="115"/>
-      <c r="D15" s="125"/>
-      <c r="E15" s="126"/>
-      <c r="F15" s="126"/>
-      <c r="G15" s="71"/>
-      <c r="H15" s="72"/>
-      <c r="I15" s="151" t="s">
-        <v>88</v>
-      </c>
-      <c r="J15" s="152"/>
-      <c r="K15" s="153"/>
+      <c r="B15" s="122"/>
+      <c r="C15" s="123"/>
+      <c r="D15" s="130"/>
+      <c r="E15" s="131"/>
+      <c r="F15" s="131"/>
+      <c r="G15" s="84"/>
+      <c r="H15" s="157"/>
+      <c r="I15" s="56" t="s">
+        <v>87</v>
+      </c>
+      <c r="J15" s="57"/>
+      <c r="K15" s="58"/>
       <c r="L15" s="30"/>
       <c r="M15" s="12">
         <v>1</v>
       </c>
-      <c r="N15" s="50" t="s">
+      <c r="N15" s="99" t="s">
         <v>47</v>
       </c>
-      <c r="O15" s="50"/>
+      <c r="O15" s="99"/>
       <c r="P15" s="5">
         <v>44895</v>
       </c>
@@ -2816,24 +2801,24 @@
     </row>
     <row r="16" spans="1:38" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>
-      <c r="B16" s="114"/>
-      <c r="C16" s="115"/>
-      <c r="D16" s="125"/>
-      <c r="E16" s="126"/>
-      <c r="F16" s="126"/>
-      <c r="G16" s="71"/>
-      <c r="H16" s="72"/>
-      <c r="I16" s="154"/>
-      <c r="J16" s="155"/>
-      <c r="K16" s="156"/>
+      <c r="B16" s="122"/>
+      <c r="C16" s="123"/>
+      <c r="D16" s="130"/>
+      <c r="E16" s="131"/>
+      <c r="F16" s="131"/>
+      <c r="G16" s="84"/>
+      <c r="H16" s="157"/>
+      <c r="I16" s="59"/>
+      <c r="J16" s="60"/>
+      <c r="K16" s="61"/>
       <c r="L16" s="30"/>
       <c r="M16" s="12">
         <v>2</v>
       </c>
-      <c r="N16" s="50" t="s">
+      <c r="N16" s="99" t="s">
         <v>47</v>
       </c>
-      <c r="O16" s="50"/>
+      <c r="O16" s="99"/>
       <c r="P16" s="5">
         <v>45107</v>
       </c>
@@ -2870,28 +2855,28 @@
     </row>
     <row r="17" spans="1:38" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="4"/>
-      <c r="B17" s="116"/>
-      <c r="C17" s="117"/>
-      <c r="D17" s="112"/>
-      <c r="E17" s="127"/>
-      <c r="F17" s="127"/>
-      <c r="G17" s="84" t="s">
+      <c r="B17" s="124"/>
+      <c r="C17" s="125"/>
+      <c r="D17" s="120"/>
+      <c r="E17" s="132"/>
+      <c r="F17" s="132"/>
+      <c r="G17" s="86" t="s">
         <v>19</v>
       </c>
-      <c r="H17" s="85"/>
-      <c r="I17" s="159" t="s">
+      <c r="H17" s="87"/>
+      <c r="I17" s="64" t="s">
         <v>20</v>
       </c>
-      <c r="J17" s="160"/>
-      <c r="K17" s="161"/>
+      <c r="J17" s="65"/>
+      <c r="K17" s="66"/>
       <c r="L17" s="30"/>
       <c r="M17" s="12">
         <v>3</v>
       </c>
-      <c r="N17" s="50" t="s">
+      <c r="N17" s="99" t="s">
         <v>47</v>
       </c>
-      <c r="O17" s="50"/>
+      <c r="O17" s="99"/>
       <c r="P17" s="5">
         <v>45473</v>
       </c>
@@ -2928,28 +2913,28 @@
     </row>
     <row r="18" spans="1:38" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="4"/>
-      <c r="B18" s="64" t="s">
+      <c r="B18" s="108" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="65"/>
-      <c r="D18" s="65"/>
-      <c r="E18" s="102"/>
-      <c r="F18" s="102"/>
-      <c r="G18" s="148" t="s">
+      <c r="C18" s="109"/>
+      <c r="D18" s="109"/>
+      <c r="E18" s="110"/>
+      <c r="F18" s="110"/>
+      <c r="G18" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="H18" s="149"/>
-      <c r="I18" s="149"/>
-      <c r="J18" s="149"/>
-      <c r="K18" s="150"/>
+      <c r="H18" s="54"/>
+      <c r="I18" s="54"/>
+      <c r="J18" s="54"/>
+      <c r="K18" s="55"/>
       <c r="L18" s="30"/>
       <c r="M18" s="13">
         <v>4</v>
       </c>
-      <c r="N18" s="42" t="s">
+      <c r="N18" s="167" t="s">
         <v>47</v>
       </c>
-      <c r="O18" s="43"/>
+      <c r="O18" s="168"/>
       <c r="P18" s="14">
         <v>45838</v>
       </c>
@@ -2986,24 +2971,24 @@
     </row>
     <row r="19" spans="1:38" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4"/>
-      <c r="B19" s="69" t="s">
+      <c r="B19" s="82" t="s">
         <v>51</v>
       </c>
-      <c r="C19" s="130"/>
-      <c r="D19" s="118" t="s">
+      <c r="C19" s="83"/>
+      <c r="D19" s="97" t="s">
         <v>52</v>
       </c>
-      <c r="E19" s="119"/>
-      <c r="F19" s="119"/>
-      <c r="G19" s="134" t="s">
+      <c r="E19" s="98"/>
+      <c r="F19" s="98"/>
+      <c r="G19" s="91" t="s">
         <v>29</v>
       </c>
-      <c r="H19" s="135"/>
-      <c r="I19" s="162" t="s">
+      <c r="H19" s="92"/>
+      <c r="I19" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="J19" s="163"/>
-      <c r="K19" s="164"/>
+      <c r="J19" s="68"/>
+      <c r="K19" s="69"/>
       <c r="L19" s="30"/>
       <c r="M19" s="30"/>
       <c r="N19" s="30"/>
@@ -3034,24 +3019,24 @@
     </row>
     <row r="20" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A20" s="4"/>
-      <c r="B20" s="71" t="s">
+      <c r="B20" s="84" t="s">
         <v>49</v>
       </c>
-      <c r="C20" s="83"/>
-      <c r="D20" s="50" t="s">
+      <c r="C20" s="85"/>
+      <c r="D20" s="99" t="s">
         <v>53</v>
       </c>
-      <c r="E20" s="120"/>
-      <c r="F20" s="120"/>
-      <c r="G20" s="51" t="s">
+      <c r="E20" s="100"/>
+      <c r="F20" s="100"/>
+      <c r="G20" s="93" t="s">
         <v>31</v>
       </c>
-      <c r="H20" s="52"/>
-      <c r="I20" s="165">
+      <c r="H20" s="94"/>
+      <c r="I20" s="70">
         <v>45636</v>
       </c>
-      <c r="J20" s="166"/>
-      <c r="K20" s="167"/>
+      <c r="J20" s="71"/>
+      <c r="K20" s="72"/>
       <c r="L20" s="30"/>
       <c r="M20" s="30"/>
       <c r="N20" s="30"/>
@@ -3082,24 +3067,24 @@
     </row>
     <row r="21" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A21" s="4"/>
-      <c r="B21" s="71" t="s">
+      <c r="B21" s="84" t="s">
         <v>50</v>
       </c>
-      <c r="C21" s="83"/>
-      <c r="D21" s="50" t="s">
+      <c r="C21" s="85"/>
+      <c r="D21" s="99" t="s">
         <v>54</v>
       </c>
-      <c r="E21" s="120"/>
-      <c r="F21" s="120"/>
-      <c r="G21" s="51" t="s">
+      <c r="E21" s="100"/>
+      <c r="F21" s="100"/>
+      <c r="G21" s="93" t="s">
         <v>30</v>
       </c>
-      <c r="H21" s="52"/>
-      <c r="I21" s="168" t="s">
+      <c r="H21" s="94"/>
+      <c r="I21" s="73" t="s">
         <v>26</v>
       </c>
-      <c r="J21" s="169"/>
-      <c r="K21" s="170"/>
+      <c r="J21" s="74"/>
+      <c r="K21" s="75"/>
       <c r="L21" s="30"/>
       <c r="M21" s="30"/>
       <c r="N21" s="30"/>
@@ -3130,24 +3115,24 @@
     </row>
     <row r="22" spans="1:38" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4"/>
-      <c r="B22" s="71" t="s">
+      <c r="B22" s="84" t="s">
         <v>66</v>
       </c>
-      <c r="C22" s="83"/>
-      <c r="D22" s="136" t="s">
+      <c r="C22" s="85"/>
+      <c r="D22" s="76" t="s">
         <v>67</v>
       </c>
-      <c r="E22" s="137"/>
-      <c r="F22" s="137"/>
-      <c r="G22" s="51" t="s">
+      <c r="E22" s="77"/>
+      <c r="F22" s="77"/>
+      <c r="G22" s="93" t="s">
         <v>28</v>
       </c>
-      <c r="H22" s="52"/>
-      <c r="I22" s="136" t="s">
+      <c r="H22" s="94"/>
+      <c r="I22" s="76" t="s">
         <v>25</v>
       </c>
-      <c r="J22" s="137"/>
-      <c r="K22" s="171"/>
+      <c r="J22" s="77"/>
+      <c r="K22" s="78"/>
       <c r="L22" s="30"/>
       <c r="M22" s="30"/>
       <c r="N22" s="30"/>
@@ -3178,20 +3163,20 @@
     </row>
     <row r="23" spans="1:38" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4"/>
-      <c r="B23" s="71" t="s">
+      <c r="B23" s="84" t="s">
         <v>68</v>
       </c>
-      <c r="C23" s="83"/>
-      <c r="D23" s="138" t="s">
+      <c r="C23" s="85"/>
+      <c r="D23" s="101" t="s">
         <v>69</v>
       </c>
-      <c r="E23" s="139"/>
-      <c r="F23" s="139"/>
-      <c r="G23" s="51"/>
-      <c r="H23" s="52"/>
-      <c r="I23" s="136"/>
-      <c r="J23" s="137"/>
-      <c r="K23" s="171"/>
+      <c r="E23" s="102"/>
+      <c r="F23" s="102"/>
+      <c r="G23" s="93"/>
+      <c r="H23" s="94"/>
+      <c r="I23" s="76"/>
+      <c r="J23" s="77"/>
+      <c r="K23" s="78"/>
       <c r="L23" s="30"/>
       <c r="M23" s="30"/>
       <c r="N23" s="30"/>
@@ -3222,20 +3207,20 @@
     </row>
     <row r="24" spans="1:38" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="4"/>
-      <c r="B24" s="84" t="s">
+      <c r="B24" s="86" t="s">
         <v>70</v>
       </c>
-      <c r="C24" s="85"/>
-      <c r="D24" s="140" t="s">
+      <c r="C24" s="87"/>
+      <c r="D24" s="103" t="s">
         <v>71</v>
       </c>
-      <c r="E24" s="141"/>
-      <c r="F24" s="141"/>
-      <c r="G24" s="98"/>
-      <c r="H24" s="75"/>
-      <c r="I24" s="172"/>
-      <c r="J24" s="173"/>
-      <c r="K24" s="174"/>
+      <c r="E24" s="104"/>
+      <c r="F24" s="104"/>
+      <c r="G24" s="95"/>
+      <c r="H24" s="96"/>
+      <c r="I24" s="79"/>
+      <c r="J24" s="80"/>
+      <c r="K24" s="81"/>
       <c r="L24" s="30"/>
       <c r="M24" s="30"/>
       <c r="N24" s="30"/>
@@ -3306,18 +3291,18 @@
     </row>
     <row r="26" spans="1:38" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4"/>
-      <c r="B26" s="142" t="s">
+      <c r="B26" s="47" t="s">
         <v>72</v>
       </c>
-      <c r="C26" s="143"/>
-      <c r="D26" s="143"/>
-      <c r="E26" s="143"/>
-      <c r="F26" s="143"/>
-      <c r="G26" s="143"/>
-      <c r="H26" s="143"/>
-      <c r="I26" s="143"/>
-      <c r="J26" s="143"/>
-      <c r="K26" s="144"/>
+      <c r="C26" s="48"/>
+      <c r="D26" s="48"/>
+      <c r="E26" s="48"/>
+      <c r="F26" s="48"/>
+      <c r="G26" s="48"/>
+      <c r="H26" s="48"/>
+      <c r="I26" s="48"/>
+      <c r="J26" s="48"/>
+      <c r="K26" s="49"/>
       <c r="L26" s="30"/>
       <c r="M26" s="30"/>
       <c r="N26" s="30"/>
@@ -3348,16 +3333,16 @@
     </row>
     <row r="27" spans="1:38" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="4"/>
-      <c r="B27" s="145"/>
-      <c r="C27" s="146"/>
-      <c r="D27" s="146"/>
-      <c r="E27" s="146"/>
-      <c r="F27" s="146"/>
-      <c r="G27" s="146"/>
-      <c r="H27" s="146"/>
-      <c r="I27" s="146"/>
-      <c r="J27" s="146"/>
-      <c r="K27" s="147"/>
+      <c r="B27" s="50"/>
+      <c r="C27" s="51"/>
+      <c r="D27" s="51"/>
+      <c r="E27" s="51"/>
+      <c r="F27" s="51"/>
+      <c r="G27" s="51"/>
+      <c r="H27" s="51"/>
+      <c r="I27" s="51"/>
+      <c r="J27" s="51"/>
+      <c r="K27" s="52"/>
       <c r="L27" s="30"/>
       <c r="M27" s="30"/>
       <c r="N27" s="30"/>
@@ -3447,7 +3432,7 @@
       <c r="B29" s="27" t="s">
         <v>76</v>
       </c>
-      <c r="C29" s="131" t="s">
+      <c r="C29" s="88" t="s">
         <v>78</v>
       </c>
       <c r="D29" s="22">
@@ -3463,7 +3448,7 @@
       <c r="G29" s="27" t="s">
         <v>76</v>
       </c>
-      <c r="H29" s="131" t="s">
+      <c r="H29" s="88" t="s">
         <v>80</v>
       </c>
       <c r="I29" s="22">
@@ -3509,7 +3494,7 @@
       <c r="B30" s="28" t="s">
         <v>77</v>
       </c>
-      <c r="C30" s="132"/>
+      <c r="C30" s="89"/>
       <c r="D30" s="5" t="s">
         <v>82</v>
       </c>
@@ -3523,7 +3508,7 @@
       <c r="G30" s="28" t="s">
         <v>77</v>
       </c>
-      <c r="H30" s="132"/>
+      <c r="H30" s="89"/>
       <c r="I30" s="5" t="s">
         <v>83</v>
       </c>
@@ -3567,7 +3552,7 @@
       <c r="B31" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="C31" s="132" t="s">
+      <c r="C31" s="89" t="s">
         <v>79</v>
       </c>
       <c r="D31" s="6">
@@ -3583,7 +3568,7 @@
       <c r="G31" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="H31" s="132" t="s">
+      <c r="H31" s="89" t="s">
         <v>81</v>
       </c>
       <c r="I31" s="6">
@@ -3629,7 +3614,7 @@
       <c r="B32" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="C32" s="133"/>
+      <c r="C32" s="90"/>
       <c r="D32" s="14" t="s">
         <v>84</v>
       </c>
@@ -3643,7 +3628,7 @@
       <c r="G32" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="H32" s="133"/>
+      <c r="H32" s="90"/>
       <c r="I32" s="21" t="s">
         <v>85</v>
       </c>
@@ -4484,20 +4469,67 @@
     </row>
   </sheetData>
   <mergeCells count="91">
-    <mergeCell ref="B26:K27"/>
-    <mergeCell ref="G18:K18"/>
-    <mergeCell ref="I15:K16"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="I19:K19"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="I22:K24"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="S10:T10"/>
+    <mergeCell ref="N18:O18"/>
+    <mergeCell ref="O6:P6"/>
+    <mergeCell ref="O7:P7"/>
+    <mergeCell ref="O8:P8"/>
+    <mergeCell ref="O9:P9"/>
+    <mergeCell ref="O10:P10"/>
+    <mergeCell ref="O11:P11"/>
+    <mergeCell ref="N15:O15"/>
+    <mergeCell ref="N16:O16"/>
+    <mergeCell ref="N17:O17"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="M10:N10"/>
+    <mergeCell ref="N14:O14"/>
+    <mergeCell ref="M13:T13"/>
+    <mergeCell ref="G13:K13"/>
+    <mergeCell ref="G14:H16"/>
+    <mergeCell ref="S11:T11"/>
+    <mergeCell ref="Q11:R11"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="M11:N11"/>
+    <mergeCell ref="Q6:R6"/>
+    <mergeCell ref="Q7:R7"/>
+    <mergeCell ref="Q8:R8"/>
+    <mergeCell ref="Q9:R9"/>
+    <mergeCell ref="Q10:R10"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="S8:T8"/>
+    <mergeCell ref="S9:T9"/>
+    <mergeCell ref="B6:F7"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="I9:K9"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B2:T2"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="M5:T5"/>
+    <mergeCell ref="B5:K5"/>
+    <mergeCell ref="B3:T3"/>
+    <mergeCell ref="B13:C17"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="D13:F17"/>
+    <mergeCell ref="G6:K7"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="G10:H10"/>
     <mergeCell ref="H29:H30"/>
     <mergeCell ref="C31:C32"/>
     <mergeCell ref="H31:H32"/>
@@ -4514,67 +4546,20 @@
     <mergeCell ref="D23:F23"/>
     <mergeCell ref="D24:F24"/>
     <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B2:T2"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="M5:T5"/>
-    <mergeCell ref="B5:K5"/>
-    <mergeCell ref="B3:T3"/>
-    <mergeCell ref="B13:C17"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="D13:F17"/>
-    <mergeCell ref="G6:K7"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="B6:F7"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="I9:K9"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="I11:K11"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="G13:K13"/>
-    <mergeCell ref="G14:H16"/>
-    <mergeCell ref="S11:T11"/>
-    <mergeCell ref="Q11:R11"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="M11:N11"/>
-    <mergeCell ref="Q6:R6"/>
-    <mergeCell ref="Q7:R7"/>
-    <mergeCell ref="Q8:R8"/>
-    <mergeCell ref="Q9:R9"/>
-    <mergeCell ref="Q10:R10"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="S8:T8"/>
-    <mergeCell ref="S9:T9"/>
-    <mergeCell ref="S10:T10"/>
-    <mergeCell ref="N18:O18"/>
-    <mergeCell ref="O6:P6"/>
-    <mergeCell ref="O7:P7"/>
-    <mergeCell ref="O8:P8"/>
-    <mergeCell ref="O9:P9"/>
-    <mergeCell ref="O10:P10"/>
-    <mergeCell ref="O11:P11"/>
-    <mergeCell ref="N15:O15"/>
-    <mergeCell ref="N16:O16"/>
-    <mergeCell ref="N17:O17"/>
-    <mergeCell ref="M8:N8"/>
-    <mergeCell ref="M9:N9"/>
-    <mergeCell ref="M10:N10"/>
-    <mergeCell ref="N14:O14"/>
-    <mergeCell ref="M13:T13"/>
+    <mergeCell ref="B26:K27"/>
+    <mergeCell ref="G18:K18"/>
+    <mergeCell ref="I15:K16"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="I17:K17"/>
+    <mergeCell ref="I19:K19"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="I21:K21"/>
+    <mergeCell ref="I22:K24"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D23" r:id="rId1" xr:uid="{0D2747F7-C52E-468D-BF9E-59F0D80A3C0A}"/>
@@ -4641,27 +4626,27 @@
     </row>
     <row r="2" spans="1:38" ht="21" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
-      <c r="B2" s="99" t="s">
-        <v>91</v>
-      </c>
-      <c r="C2" s="100"/>
-      <c r="D2" s="100"/>
-      <c r="E2" s="100"/>
-      <c r="F2" s="100"/>
-      <c r="G2" s="100"/>
-      <c r="H2" s="100"/>
-      <c r="I2" s="100"/>
-      <c r="J2" s="100"/>
-      <c r="K2" s="100"/>
-      <c r="L2" s="100"/>
-      <c r="M2" s="100"/>
-      <c r="N2" s="100"/>
-      <c r="O2" s="100"/>
-      <c r="P2" s="100"/>
-      <c r="Q2" s="100"/>
-      <c r="R2" s="100"/>
-      <c r="S2" s="100"/>
-      <c r="T2" s="101"/>
+      <c r="B2" s="105" t="s">
+        <v>90</v>
+      </c>
+      <c r="C2" s="106"/>
+      <c r="D2" s="106"/>
+      <c r="E2" s="106"/>
+      <c r="F2" s="106"/>
+      <c r="G2" s="106"/>
+      <c r="H2" s="106"/>
+      <c r="I2" s="106"/>
+      <c r="J2" s="106"/>
+      <c r="K2" s="106"/>
+      <c r="L2" s="106"/>
+      <c r="M2" s="106"/>
+      <c r="N2" s="106"/>
+      <c r="O2" s="106"/>
+      <c r="P2" s="106"/>
+      <c r="Q2" s="106"/>
+      <c r="R2" s="106"/>
+      <c r="S2" s="106"/>
+      <c r="T2" s="107"/>
       <c r="U2" s="4"/>
       <c r="V2" s="4"/>
       <c r="W2" s="4"/>
@@ -4683,27 +4668,27 @@
     </row>
     <row r="3" spans="1:38" ht="40.799999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2"/>
-      <c r="B3" s="110" t="s">
+      <c r="B3" s="118" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="111"/>
-      <c r="D3" s="111"/>
-      <c r="E3" s="111"/>
-      <c r="F3" s="111"/>
-      <c r="G3" s="112"/>
-      <c r="H3" s="112"/>
-      <c r="I3" s="112"/>
-      <c r="J3" s="112"/>
-      <c r="K3" s="112"/>
-      <c r="L3" s="112"/>
-      <c r="M3" s="112"/>
-      <c r="N3" s="112"/>
-      <c r="O3" s="112"/>
-      <c r="P3" s="112"/>
-      <c r="Q3" s="112"/>
-      <c r="R3" s="112"/>
-      <c r="S3" s="112"/>
-      <c r="T3" s="113"/>
+      <c r="C3" s="119"/>
+      <c r="D3" s="119"/>
+      <c r="E3" s="119"/>
+      <c r="F3" s="119"/>
+      <c r="G3" s="120"/>
+      <c r="H3" s="120"/>
+      <c r="I3" s="120"/>
+      <c r="J3" s="120"/>
+      <c r="K3" s="120"/>
+      <c r="L3" s="120"/>
+      <c r="M3" s="120"/>
+      <c r="N3" s="120"/>
+      <c r="O3" s="120"/>
+      <c r="P3" s="120"/>
+      <c r="Q3" s="120"/>
+      <c r="R3" s="120"/>
+      <c r="S3" s="120"/>
+      <c r="T3" s="121"/>
       <c r="U3" s="4"/>
       <c r="V3" s="4"/>
       <c r="W3" s="4"/>
@@ -4765,29 +4750,29 @@
     </row>
     <row r="5" spans="1:38" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4"/>
-      <c r="B5" s="106" t="s">
+      <c r="B5" s="114" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="107"/>
-      <c r="D5" s="107"/>
-      <c r="E5" s="107"/>
-      <c r="F5" s="107"/>
-      <c r="G5" s="107"/>
-      <c r="H5" s="107"/>
-      <c r="I5" s="107"/>
-      <c r="J5" s="108"/>
-      <c r="K5" s="109"/>
+      <c r="C5" s="115"/>
+      <c r="D5" s="115"/>
+      <c r="E5" s="115"/>
+      <c r="F5" s="115"/>
+      <c r="G5" s="115"/>
+      <c r="H5" s="115"/>
+      <c r="I5" s="115"/>
+      <c r="J5" s="116"/>
+      <c r="K5" s="117"/>
       <c r="L5" s="19"/>
-      <c r="M5" s="103" t="s">
+      <c r="M5" s="111" t="s">
         <v>27</v>
       </c>
-      <c r="N5" s="104"/>
-      <c r="O5" s="104"/>
-      <c r="P5" s="104"/>
-      <c r="Q5" s="104"/>
-      <c r="R5" s="104"/>
-      <c r="S5" s="104"/>
-      <c r="T5" s="105"/>
+      <c r="N5" s="112"/>
+      <c r="O5" s="112"/>
+      <c r="P5" s="112"/>
+      <c r="Q5" s="112"/>
+      <c r="R5" s="112"/>
+      <c r="S5" s="112"/>
+      <c r="T5" s="113"/>
       <c r="U5" s="4"/>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
@@ -4809,37 +4794,37 @@
     </row>
     <row r="6" spans="1:38" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="18"/>
-      <c r="B6" s="77" t="s">
+      <c r="B6" s="133" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="78"/>
-      <c r="D6" s="78"/>
-      <c r="E6" s="79"/>
-      <c r="F6" s="128"/>
-      <c r="G6" s="77" t="s">
+      <c r="C6" s="134"/>
+      <c r="D6" s="134"/>
+      <c r="E6" s="135"/>
+      <c r="F6" s="136"/>
+      <c r="G6" s="133" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="78"/>
-      <c r="I6" s="78"/>
-      <c r="J6" s="79"/>
-      <c r="K6" s="128"/>
+      <c r="H6" s="134"/>
+      <c r="I6" s="134"/>
+      <c r="J6" s="135"/>
+      <c r="K6" s="136"/>
       <c r="L6" s="20"/>
-      <c r="M6" s="51" t="s">
+      <c r="M6" s="93" t="s">
         <v>39</v>
       </c>
-      <c r="N6" s="52"/>
-      <c r="O6" s="44" t="s">
+      <c r="N6" s="94"/>
+      <c r="O6" s="169" t="s">
         <v>59</v>
       </c>
-      <c r="P6" s="44"/>
-      <c r="Q6" s="57" t="s">
+      <c r="P6" s="169"/>
+      <c r="Q6" s="161" t="s">
         <v>37</v>
       </c>
-      <c r="R6" s="57"/>
-      <c r="S6" s="53">
+      <c r="R6" s="161"/>
+      <c r="S6" s="163">
         <v>1252370.6000000001</v>
       </c>
-      <c r="T6" s="54"/>
+      <c r="T6" s="164"/>
       <c r="U6" s="18"/>
       <c r="V6" s="18"/>
       <c r="W6" s="18"/>
@@ -4861,33 +4846,33 @@
     </row>
     <row r="7" spans="1:38" s="1" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="18"/>
-      <c r="B7" s="80"/>
-      <c r="C7" s="81"/>
-      <c r="D7" s="81"/>
-      <c r="E7" s="82"/>
-      <c r="F7" s="129"/>
-      <c r="G7" s="80"/>
-      <c r="H7" s="81"/>
-      <c r="I7" s="81"/>
-      <c r="J7" s="82"/>
-      <c r="K7" s="129"/>
+      <c r="B7" s="137"/>
+      <c r="C7" s="138"/>
+      <c r="D7" s="138"/>
+      <c r="E7" s="139"/>
+      <c r="F7" s="140"/>
+      <c r="G7" s="137"/>
+      <c r="H7" s="138"/>
+      <c r="I7" s="138"/>
+      <c r="J7" s="139"/>
+      <c r="K7" s="140"/>
       <c r="L7" s="20"/>
-      <c r="M7" s="51" t="s">
+      <c r="M7" s="93" t="s">
         <v>32</v>
       </c>
-      <c r="N7" s="76"/>
-      <c r="O7" s="175" t="s">
+      <c r="N7" s="160"/>
+      <c r="O7" s="199" t="s">
         <v>60</v>
       </c>
-      <c r="P7" s="176"/>
-      <c r="Q7" s="58" t="s">
+      <c r="P7" s="200"/>
+      <c r="Q7" s="162" t="s">
         <v>55</v>
       </c>
-      <c r="R7" s="52"/>
-      <c r="S7" s="53" t="s">
+      <c r="R7" s="94"/>
+      <c r="S7" s="163" t="s">
         <v>65</v>
       </c>
-      <c r="T7" s="54"/>
+      <c r="T7" s="164"/>
       <c r="U7" s="18"/>
       <c r="V7" s="18"/>
       <c r="W7" s="18"/>
@@ -4909,41 +4894,41 @@
     </row>
     <row r="8" spans="1:38" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
-      <c r="B8" s="69" t="s">
+      <c r="B8" s="82" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="130"/>
-      <c r="D8" s="118" t="s">
-        <v>92</v>
-      </c>
-      <c r="E8" s="119"/>
+      <c r="C8" s="83"/>
+      <c r="D8" s="97" t="s">
+        <v>91</v>
+      </c>
+      <c r="E8" s="98"/>
       <c r="F8" s="187"/>
-      <c r="G8" s="69" t="s">
+      <c r="G8" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="H8" s="130"/>
-      <c r="I8" s="86" t="s">
-        <v>98</v>
-      </c>
-      <c r="J8" s="87"/>
-      <c r="K8" s="88"/>
+      <c r="H8" s="83"/>
+      <c r="I8" s="141" t="s">
+        <v>97</v>
+      </c>
+      <c r="J8" s="142"/>
+      <c r="K8" s="143"/>
       <c r="L8" s="19"/>
-      <c r="M8" s="51" t="s">
+      <c r="M8" s="93" t="s">
         <v>33</v>
       </c>
-      <c r="N8" s="52"/>
-      <c r="O8" s="177" t="s">
+      <c r="N8" s="94"/>
+      <c r="O8" s="198" t="s">
         <v>61</v>
       </c>
-      <c r="P8" s="177"/>
-      <c r="Q8" s="52" t="s">
+      <c r="P8" s="198"/>
+      <c r="Q8" s="94" t="s">
         <v>56</v>
       </c>
-      <c r="R8" s="52"/>
-      <c r="S8" s="55">
+      <c r="R8" s="94"/>
+      <c r="S8" s="165">
         <v>44517</v>
       </c>
-      <c r="T8" s="56"/>
+      <c r="T8" s="166"/>
       <c r="U8" s="4"/>
       <c r="V8" s="4"/>
       <c r="W8" s="4"/>
@@ -4965,41 +4950,41 @@
     </row>
     <row r="9" spans="1:38" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
-      <c r="B9" s="71" t="s">
+      <c r="B9" s="84" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="83"/>
-      <c r="D9" s="50" t="s">
-        <v>93</v>
-      </c>
-      <c r="E9" s="120"/>
-      <c r="F9" s="188"/>
-      <c r="G9" s="71" t="s">
+      <c r="C9" s="85"/>
+      <c r="D9" s="99" t="s">
+        <v>92</v>
+      </c>
+      <c r="E9" s="100"/>
+      <c r="F9" s="181"/>
+      <c r="G9" s="84" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="83"/>
-      <c r="I9" s="89">
+      <c r="H9" s="85"/>
+      <c r="I9" s="144">
         <v>45964</v>
       </c>
-      <c r="J9" s="90"/>
-      <c r="K9" s="91"/>
+      <c r="J9" s="145"/>
+      <c r="K9" s="146"/>
       <c r="L9" s="19"/>
-      <c r="M9" s="51" t="s">
+      <c r="M9" s="93" t="s">
         <v>34</v>
       </c>
-      <c r="N9" s="52"/>
-      <c r="O9" s="48" t="s">
+      <c r="N9" s="94"/>
+      <c r="O9" s="171" t="s">
         <v>62</v>
       </c>
-      <c r="P9" s="48"/>
-      <c r="Q9" s="52" t="s">
+      <c r="P9" s="171"/>
+      <c r="Q9" s="94" t="s">
         <v>15</v>
       </c>
-      <c r="R9" s="52"/>
-      <c r="S9" s="55">
+      <c r="R9" s="94"/>
+      <c r="S9" s="165">
         <v>44511</v>
       </c>
-      <c r="T9" s="56"/>
+      <c r="T9" s="166"/>
       <c r="U9" s="4"/>
       <c r="V9" s="4"/>
       <c r="W9" s="4"/>
@@ -5021,41 +5006,41 @@
     </row>
     <row r="10" spans="1:38" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
-      <c r="B10" s="71" t="s">
+      <c r="B10" s="84" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="83"/>
-      <c r="D10" s="121">
+      <c r="C10" s="85"/>
+      <c r="D10" s="126">
         <v>45961</v>
       </c>
-      <c r="E10" s="122"/>
-      <c r="F10" s="189"/>
-      <c r="G10" s="71" t="s">
+      <c r="E10" s="127"/>
+      <c r="F10" s="197"/>
+      <c r="G10" s="84" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="83"/>
-      <c r="I10" s="92">
+      <c r="H10" s="85"/>
+      <c r="I10" s="147">
         <v>457556.31</v>
       </c>
-      <c r="J10" s="93"/>
-      <c r="K10" s="94"/>
+      <c r="J10" s="148"/>
+      <c r="K10" s="149"/>
       <c r="L10" s="19"/>
-      <c r="M10" s="51" t="s">
+      <c r="M10" s="93" t="s">
         <v>35</v>
       </c>
-      <c r="N10" s="52"/>
-      <c r="O10" s="48" t="s">
+      <c r="N10" s="94"/>
+      <c r="O10" s="171" t="s">
         <v>63</v>
       </c>
-      <c r="P10" s="48"/>
-      <c r="Q10" s="52" t="s">
+      <c r="P10" s="171"/>
+      <c r="Q10" s="94" t="s">
         <v>16</v>
       </c>
-      <c r="R10" s="52"/>
-      <c r="S10" s="55">
+      <c r="R10" s="94"/>
+      <c r="S10" s="165">
         <v>44895</v>
       </c>
-      <c r="T10" s="56"/>
+      <c r="T10" s="166"/>
       <c r="U10" s="4"/>
       <c r="V10" s="4"/>
       <c r="W10" s="4"/>
@@ -5077,41 +5062,41 @@
     </row>
     <row r="11" spans="1:38" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4"/>
-      <c r="B11" s="71" t="s">
+      <c r="B11" s="84" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="83"/>
-      <c r="D11" s="123">
+      <c r="C11" s="85"/>
+      <c r="D11" s="128">
         <v>457556.31</v>
       </c>
-      <c r="E11" s="124"/>
-      <c r="F11" s="190"/>
-      <c r="G11" s="71" t="s">
+      <c r="E11" s="129"/>
+      <c r="F11" s="194"/>
+      <c r="G11" s="84" t="s">
         <v>15</v>
       </c>
-      <c r="H11" s="83"/>
-      <c r="I11" s="89">
+      <c r="H11" s="85"/>
+      <c r="I11" s="144">
         <v>45964</v>
       </c>
-      <c r="J11" s="90"/>
-      <c r="K11" s="91"/>
+      <c r="J11" s="145"/>
+      <c r="K11" s="146"/>
       <c r="L11" s="19"/>
-      <c r="M11" s="98" t="s">
+      <c r="M11" s="95" t="s">
         <v>36</v>
       </c>
-      <c r="N11" s="75"/>
-      <c r="O11" s="49" t="s">
+      <c r="N11" s="96"/>
+      <c r="O11" s="172" t="s">
         <v>64</v>
       </c>
-      <c r="P11" s="49"/>
-      <c r="Q11" s="75" t="s">
+      <c r="P11" s="172"/>
+      <c r="Q11" s="96" t="s">
         <v>57</v>
       </c>
-      <c r="R11" s="75"/>
-      <c r="S11" s="73">
+      <c r="R11" s="96"/>
+      <c r="S11" s="158">
         <v>0</v>
       </c>
-      <c r="T11" s="74"/>
+      <c r="T11" s="159"/>
       <c r="U11" s="4"/>
       <c r="V11" s="4"/>
       <c r="W11" s="4"/>
@@ -5133,24 +5118,24 @@
     </row>
     <row r="12" spans="1:38" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4"/>
-      <c r="B12" s="71" t="s">
+      <c r="B12" s="84" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="83"/>
-      <c r="D12" s="123" t="s">
-        <v>90</v>
-      </c>
-      <c r="E12" s="124"/>
-      <c r="F12" s="190"/>
-      <c r="G12" s="84" t="s">
+      <c r="C12" s="85"/>
+      <c r="D12" s="128" t="s">
+        <v>89</v>
+      </c>
+      <c r="E12" s="129"/>
+      <c r="F12" s="194"/>
+      <c r="G12" s="86" t="s">
         <v>16</v>
       </c>
-      <c r="H12" s="85"/>
-      <c r="I12" s="95">
+      <c r="H12" s="87"/>
+      <c r="I12" s="150">
         <v>46268</v>
       </c>
-      <c r="J12" s="96"/>
-      <c r="K12" s="97"/>
+      <c r="J12" s="151"/>
+      <c r="K12" s="152"/>
       <c r="L12" s="19"/>
       <c r="M12" s="8" t="s">
         <v>38</v>
@@ -5183,33 +5168,33 @@
     </row>
     <row r="13" spans="1:38" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4"/>
-      <c r="B13" s="114" t="s">
+      <c r="B13" s="122" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="115"/>
-      <c r="D13" s="125" t="s">
+      <c r="C13" s="123"/>
+      <c r="D13" s="130" t="s">
         <v>58</v>
       </c>
-      <c r="E13" s="126"/>
-      <c r="F13" s="191"/>
-      <c r="G13" s="64" t="s">
+      <c r="E13" s="131"/>
+      <c r="F13" s="195"/>
+      <c r="G13" s="108" t="s">
         <v>17</v>
       </c>
-      <c r="H13" s="65"/>
-      <c r="I13" s="65"/>
-      <c r="J13" s="102"/>
-      <c r="K13" s="192"/>
+      <c r="H13" s="109"/>
+      <c r="I13" s="109"/>
+      <c r="J13" s="110"/>
+      <c r="K13" s="185"/>
       <c r="L13" s="30"/>
-      <c r="M13" s="61" t="s">
+      <c r="M13" s="175" t="s">
         <v>38</v>
       </c>
-      <c r="N13" s="62"/>
-      <c r="O13" s="62"/>
-      <c r="P13" s="62"/>
-      <c r="Q13" s="62"/>
-      <c r="R13" s="62"/>
-      <c r="S13" s="62"/>
-      <c r="T13" s="63"/>
+      <c r="N13" s="176"/>
+      <c r="O13" s="176"/>
+      <c r="P13" s="176"/>
+      <c r="Q13" s="176"/>
+      <c r="R13" s="176"/>
+      <c r="S13" s="176"/>
+      <c r="T13" s="177"/>
       <c r="U13" s="4"/>
       <c r="V13" s="4"/>
       <c r="W13" s="4"/>
@@ -5231,28 +5216,28 @@
     </row>
     <row r="14" spans="1:38" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="4"/>
-      <c r="B14" s="114"/>
-      <c r="C14" s="115"/>
-      <c r="D14" s="125"/>
-      <c r="E14" s="126"/>
-      <c r="F14" s="191"/>
-      <c r="G14" s="194" t="s">
+      <c r="B14" s="122"/>
+      <c r="C14" s="123"/>
+      <c r="D14" s="130"/>
+      <c r="E14" s="131"/>
+      <c r="F14" s="195"/>
+      <c r="G14" s="192" t="s">
         <v>18</v>
       </c>
-      <c r="H14" s="195"/>
-      <c r="I14" s="196" t="s">
-        <v>99</v>
-      </c>
-      <c r="J14" s="196"/>
-      <c r="K14" s="197"/>
+      <c r="H14" s="193"/>
+      <c r="I14" s="190" t="s">
+        <v>98</v>
+      </c>
+      <c r="J14" s="190"/>
+      <c r="K14" s="191"/>
       <c r="L14" s="30"/>
       <c r="M14" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="N14" s="59" t="s">
+      <c r="N14" s="173" t="s">
         <v>41</v>
       </c>
-      <c r="O14" s="60"/>
+      <c r="O14" s="174"/>
       <c r="P14" s="7" t="s">
         <v>42</v>
       </c>
@@ -5289,24 +5274,24 @@
     </row>
     <row r="15" spans="1:38" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4"/>
-      <c r="B15" s="114"/>
-      <c r="C15" s="115"/>
-      <c r="D15" s="125"/>
-      <c r="E15" s="126"/>
-      <c r="F15" s="191"/>
-      <c r="G15" s="179"/>
-      <c r="H15" s="179"/>
-      <c r="I15" s="180"/>
-      <c r="J15" s="180"/>
-      <c r="K15" s="180"/>
+      <c r="B15" s="122"/>
+      <c r="C15" s="123"/>
+      <c r="D15" s="130"/>
+      <c r="E15" s="131"/>
+      <c r="F15" s="195"/>
+      <c r="G15" s="42"/>
+      <c r="H15" s="42"/>
+      <c r="I15" s="189"/>
+      <c r="J15" s="189"/>
+      <c r="K15" s="189"/>
       <c r="L15" s="30"/>
       <c r="M15" s="12">
         <v>1</v>
       </c>
-      <c r="N15" s="50" t="s">
+      <c r="N15" s="99" t="s">
         <v>47</v>
       </c>
-      <c r="O15" s="50"/>
+      <c r="O15" s="99"/>
       <c r="P15" s="40">
         <v>44895</v>
       </c>
@@ -5343,24 +5328,24 @@
     </row>
     <row r="16" spans="1:38" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>
-      <c r="B16" s="114"/>
-      <c r="C16" s="115"/>
-      <c r="D16" s="125"/>
-      <c r="E16" s="126"/>
-      <c r="F16" s="191"/>
-      <c r="G16" s="179"/>
-      <c r="H16" s="179"/>
-      <c r="I16" s="180"/>
-      <c r="J16" s="180"/>
-      <c r="K16" s="180"/>
+      <c r="B16" s="122"/>
+      <c r="C16" s="123"/>
+      <c r="D16" s="130"/>
+      <c r="E16" s="131"/>
+      <c r="F16" s="195"/>
+      <c r="G16" s="42"/>
+      <c r="H16" s="42"/>
+      <c r="I16" s="189"/>
+      <c r="J16" s="189"/>
+      <c r="K16" s="189"/>
       <c r="L16" s="30"/>
       <c r="M16" s="12">
         <v>2</v>
       </c>
-      <c r="N16" s="50" t="s">
+      <c r="N16" s="99" t="s">
         <v>47</v>
       </c>
-      <c r="O16" s="50"/>
+      <c r="O16" s="99"/>
       <c r="P16" s="40">
         <v>45107</v>
       </c>
@@ -5397,24 +5382,24 @@
     </row>
     <row r="17" spans="1:38" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="4"/>
-      <c r="B17" s="116"/>
-      <c r="C17" s="117"/>
-      <c r="D17" s="112"/>
-      <c r="E17" s="127"/>
-      <c r="F17" s="113"/>
-      <c r="G17" s="181"/>
-      <c r="H17" s="181"/>
-      <c r="I17" s="182"/>
-      <c r="J17" s="182"/>
-      <c r="K17" s="182"/>
+      <c r="B17" s="124"/>
+      <c r="C17" s="125"/>
+      <c r="D17" s="120"/>
+      <c r="E17" s="132"/>
+      <c r="F17" s="121"/>
+      <c r="G17" s="178"/>
+      <c r="H17" s="178"/>
+      <c r="I17" s="196"/>
+      <c r="J17" s="196"/>
+      <c r="K17" s="196"/>
       <c r="L17" s="30"/>
       <c r="M17" s="12">
         <v>3</v>
       </c>
-      <c r="N17" s="50" t="s">
+      <c r="N17" s="99" t="s">
         <v>47</v>
       </c>
-      <c r="O17" s="50"/>
+      <c r="O17" s="99"/>
       <c r="P17" s="40">
         <v>45473</v>
       </c>
@@ -5451,26 +5436,26 @@
     </row>
     <row r="18" spans="1:38" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="4"/>
-      <c r="B18" s="64" t="s">
+      <c r="B18" s="108" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="65"/>
-      <c r="D18" s="65"/>
-      <c r="E18" s="102"/>
-      <c r="F18" s="192"/>
-      <c r="G18" s="183"/>
-      <c r="H18" s="183"/>
-      <c r="I18" s="183"/>
-      <c r="J18" s="183"/>
-      <c r="K18" s="183"/>
+      <c r="C18" s="109"/>
+      <c r="D18" s="109"/>
+      <c r="E18" s="110"/>
+      <c r="F18" s="185"/>
+      <c r="G18" s="186"/>
+      <c r="H18" s="186"/>
+      <c r="I18" s="186"/>
+      <c r="J18" s="186"/>
+      <c r="K18" s="186"/>
       <c r="L18" s="30"/>
       <c r="M18" s="12">
         <v>4</v>
       </c>
-      <c r="N18" s="50" t="s">
+      <c r="N18" s="99" t="s">
         <v>47</v>
       </c>
-      <c r="O18" s="50"/>
+      <c r="O18" s="99"/>
       <c r="P18" s="40">
         <v>45838</v>
       </c>
@@ -5507,41 +5492,41 @@
     </row>
     <row r="19" spans="1:38" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="4"/>
-      <c r="B19" s="69" t="s">
+      <c r="B19" s="82" t="s">
         <v>51</v>
       </c>
-      <c r="C19" s="130"/>
-      <c r="D19" s="118" t="s">
-        <v>94</v>
-      </c>
-      <c r="E19" s="119"/>
+      <c r="C19" s="83"/>
+      <c r="D19" s="97" t="s">
+        <v>93</v>
+      </c>
+      <c r="E19" s="98"/>
       <c r="F19" s="187"/>
-      <c r="G19" s="181"/>
-      <c r="H19" s="181"/>
+      <c r="G19" s="178"/>
+      <c r="H19" s="178"/>
       <c r="I19" s="184"/>
       <c r="J19" s="184"/>
       <c r="K19" s="184"/>
       <c r="L19" s="30"/>
-      <c r="M19" s="198">
+      <c r="M19" s="43">
         <v>5</v>
       </c>
-      <c r="N19" s="160" t="s">
+      <c r="N19" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="O19" s="199"/>
-      <c r="P19" s="200">
+      <c r="O19" s="188"/>
+      <c r="P19" s="44">
         <v>46203</v>
       </c>
-      <c r="Q19" s="200">
+      <c r="Q19" s="44">
         <v>46568</v>
       </c>
-      <c r="R19" s="201">
+      <c r="R19" s="45">
         <v>0</v>
       </c>
-      <c r="S19" s="201">
+      <c r="S19" s="45">
         <v>0</v>
       </c>
-      <c r="T19" s="202">
+      <c r="T19" s="46">
         <v>0</v>
       </c>
       <c r="U19" s="4"/>
@@ -5565,20 +5550,20 @@
     </row>
     <row r="20" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A20" s="4"/>
-      <c r="B20" s="71" t="s">
+      <c r="B20" s="84" t="s">
         <v>49</v>
       </c>
-      <c r="C20" s="83"/>
-      <c r="D20" s="50" t="s">
-        <v>95</v>
-      </c>
-      <c r="E20" s="120"/>
-      <c r="F20" s="188"/>
-      <c r="G20" s="181"/>
-      <c r="H20" s="181"/>
-      <c r="I20" s="185"/>
-      <c r="J20" s="185"/>
-      <c r="K20" s="185"/>
+      <c r="C20" s="85"/>
+      <c r="D20" s="99" t="s">
+        <v>94</v>
+      </c>
+      <c r="E20" s="100"/>
+      <c r="F20" s="181"/>
+      <c r="G20" s="178"/>
+      <c r="H20" s="178"/>
+      <c r="I20" s="182"/>
+      <c r="J20" s="182"/>
+      <c r="K20" s="182"/>
       <c r="L20" s="30"/>
       <c r="M20" s="30"/>
       <c r="N20" s="30"/>
@@ -5609,17 +5594,17 @@
     </row>
     <row r="21" spans="1:38" x14ac:dyDescent="0.3">
       <c r="A21" s="4"/>
-      <c r="B21" s="71" t="s">
+      <c r="B21" s="84" t="s">
         <v>50</v>
       </c>
-      <c r="C21" s="83"/>
-      <c r="D21" s="178" t="s">
-        <v>96</v>
-      </c>
-      <c r="E21" s="120"/>
-      <c r="F21" s="188"/>
-      <c r="G21" s="181"/>
-      <c r="H21" s="181"/>
+      <c r="C21" s="85"/>
+      <c r="D21" s="183" t="s">
+        <v>95</v>
+      </c>
+      <c r="E21" s="100"/>
+      <c r="F21" s="181"/>
+      <c r="G21" s="178"/>
+      <c r="H21" s="178"/>
       <c r="I21" s="184"/>
       <c r="J21" s="184"/>
       <c r="K21" s="184"/>
@@ -5653,20 +5638,20 @@
     </row>
     <row r="22" spans="1:38" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4"/>
-      <c r="B22" s="71" t="s">
+      <c r="B22" s="84" t="s">
         <v>66</v>
       </c>
-      <c r="C22" s="83"/>
-      <c r="D22" s="136" t="s">
-        <v>97</v>
-      </c>
-      <c r="E22" s="137"/>
-      <c r="F22" s="171"/>
-      <c r="G22" s="181"/>
-      <c r="H22" s="181"/>
-      <c r="I22" s="186"/>
-      <c r="J22" s="186"/>
-      <c r="K22" s="186"/>
+      <c r="C22" s="85"/>
+      <c r="D22" s="76" t="s">
+        <v>96</v>
+      </c>
+      <c r="E22" s="77"/>
+      <c r="F22" s="78"/>
+      <c r="G22" s="178"/>
+      <c r="H22" s="178"/>
+      <c r="I22" s="179"/>
+      <c r="J22" s="179"/>
+      <c r="K22" s="179"/>
       <c r="L22" s="30"/>
       <c r="M22" s="30"/>
       <c r="N22" s="30"/>
@@ -5697,20 +5682,20 @@
     </row>
     <row r="23" spans="1:38" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4"/>
-      <c r="B23" s="71" t="s">
+      <c r="B23" s="84" t="s">
         <v>68</v>
       </c>
-      <c r="C23" s="83"/>
-      <c r="D23" s="136" t="s">
-        <v>90</v>
-      </c>
-      <c r="E23" s="137"/>
-      <c r="F23" s="171"/>
-      <c r="G23" s="181"/>
-      <c r="H23" s="181"/>
-      <c r="I23" s="186"/>
-      <c r="J23" s="186"/>
-      <c r="K23" s="186"/>
+      <c r="C23" s="85"/>
+      <c r="D23" s="76" t="s">
+        <v>89</v>
+      </c>
+      <c r="E23" s="77"/>
+      <c r="F23" s="78"/>
+      <c r="G23" s="178"/>
+      <c r="H23" s="178"/>
+      <c r="I23" s="179"/>
+      <c r="J23" s="179"/>
+      <c r="K23" s="179"/>
       <c r="L23" s="30"/>
       <c r="M23" s="30"/>
       <c r="N23" s="30"/>
@@ -5741,20 +5726,20 @@
     </row>
     <row r="24" spans="1:38" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="4"/>
-      <c r="B24" s="84" t="s">
+      <c r="B24" s="86" t="s">
         <v>70</v>
       </c>
-      <c r="C24" s="85"/>
-      <c r="D24" s="140" t="s">
-        <v>90</v>
-      </c>
-      <c r="E24" s="141"/>
-      <c r="F24" s="193"/>
-      <c r="G24" s="181"/>
-      <c r="H24" s="181"/>
-      <c r="I24" s="186"/>
-      <c r="J24" s="186"/>
-      <c r="K24" s="186"/>
+      <c r="C24" s="87"/>
+      <c r="D24" s="103" t="s">
+        <v>89</v>
+      </c>
+      <c r="E24" s="104"/>
+      <c r="F24" s="180"/>
+      <c r="G24" s="178"/>
+      <c r="H24" s="178"/>
+      <c r="I24" s="179"/>
+      <c r="J24" s="179"/>
+      <c r="K24" s="179"/>
       <c r="L24" s="30"/>
       <c r="M24" s="30"/>
       <c r="N24" s="30"/>
@@ -5825,18 +5810,18 @@
     </row>
     <row r="26" spans="1:38" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4"/>
-      <c r="B26" s="142" t="s">
+      <c r="B26" s="47" t="s">
         <v>72</v>
       </c>
-      <c r="C26" s="143"/>
-      <c r="D26" s="143"/>
-      <c r="E26" s="143"/>
-      <c r="F26" s="143"/>
-      <c r="G26" s="143"/>
-      <c r="H26" s="143"/>
-      <c r="I26" s="143"/>
-      <c r="J26" s="143"/>
-      <c r="K26" s="144"/>
+      <c r="C26" s="48"/>
+      <c r="D26" s="48"/>
+      <c r="E26" s="48"/>
+      <c r="F26" s="48"/>
+      <c r="G26" s="48"/>
+      <c r="H26" s="48"/>
+      <c r="I26" s="48"/>
+      <c r="J26" s="48"/>
+      <c r="K26" s="49"/>
       <c r="L26" s="30"/>
       <c r="M26" s="30"/>
       <c r="N26" s="30"/>
@@ -5867,16 +5852,16 @@
     </row>
     <row r="27" spans="1:38" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="4"/>
-      <c r="B27" s="145"/>
-      <c r="C27" s="146"/>
-      <c r="D27" s="146"/>
-      <c r="E27" s="146"/>
-      <c r="F27" s="146"/>
-      <c r="G27" s="146"/>
-      <c r="H27" s="146"/>
-      <c r="I27" s="146"/>
-      <c r="J27" s="146"/>
-      <c r="K27" s="147"/>
+      <c r="B27" s="50"/>
+      <c r="C27" s="51"/>
+      <c r="D27" s="51"/>
+      <c r="E27" s="51"/>
+      <c r="F27" s="51"/>
+      <c r="G27" s="51"/>
+      <c r="H27" s="51"/>
+      <c r="I27" s="51"/>
+      <c r="J27" s="51"/>
+      <c r="K27" s="52"/>
       <c r="L27" s="30"/>
       <c r="M27" s="30"/>
       <c r="N27" s="30"/>
@@ -5966,7 +5951,7 @@
       <c r="B29" s="27" t="s">
         <v>76</v>
       </c>
-      <c r="C29" s="131" t="s">
+      <c r="C29" s="88" t="s">
         <v>78</v>
       </c>
       <c r="D29" s="22">
@@ -5982,7 +5967,7 @@
       <c r="G29" s="27" t="s">
         <v>76</v>
       </c>
-      <c r="H29" s="131" t="s">
+      <c r="H29" s="88" t="s">
         <v>80</v>
       </c>
       <c r="I29" s="22">
@@ -6028,9 +6013,9 @@
       <c r="B30" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="C30" s="133"/>
+      <c r="C30" s="90"/>
       <c r="D30" s="14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E30" s="14">
         <v>46003</v>
@@ -6042,9 +6027,9 @@
       <c r="G30" s="29" t="s">
         <v>77</v>
       </c>
-      <c r="H30" s="133"/>
+      <c r="H30" s="90"/>
       <c r="I30" s="14" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J30" s="14">
         <v>46302</v>
@@ -6883,50 +6868,36 @@
     </row>
   </sheetData>
   <mergeCells count="90">
-    <mergeCell ref="B26:K27"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="H29:H30"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="G22:H24"/>
-    <mergeCell ref="I22:K24"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="D24:F24"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="D21:F21"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="I21:K21"/>
-    <mergeCell ref="N17:O17"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="G18:K18"/>
-    <mergeCell ref="N18:O18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="I19:K19"/>
-    <mergeCell ref="N19:O19"/>
-    <mergeCell ref="M13:T13"/>
-    <mergeCell ref="N14:O14"/>
-    <mergeCell ref="I15:K16"/>
-    <mergeCell ref="N15:O15"/>
-    <mergeCell ref="N16:O16"/>
-    <mergeCell ref="I14:K14"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="B13:C17"/>
-    <mergeCell ref="D13:F17"/>
-    <mergeCell ref="G13:K13"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="I17:K17"/>
+    <mergeCell ref="B2:T2"/>
+    <mergeCell ref="B3:T3"/>
+    <mergeCell ref="B5:K5"/>
+    <mergeCell ref="M5:T5"/>
+    <mergeCell ref="B6:F7"/>
+    <mergeCell ref="G6:K7"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="O6:P6"/>
+    <mergeCell ref="Q6:R6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="O7:P7"/>
+    <mergeCell ref="Q7:R7"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="O8:P8"/>
+    <mergeCell ref="Q8:R8"/>
+    <mergeCell ref="S8:T8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="I9:K9"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="O9:P9"/>
+    <mergeCell ref="Q9:R9"/>
+    <mergeCell ref="S9:T9"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="M8:N8"/>
     <mergeCell ref="Q10:R10"/>
     <mergeCell ref="S10:T10"/>
     <mergeCell ref="B11:C11"/>
@@ -6943,36 +6914,50 @@
     <mergeCell ref="I10:K10"/>
     <mergeCell ref="M10:N10"/>
     <mergeCell ref="O10:P10"/>
-    <mergeCell ref="O8:P8"/>
-    <mergeCell ref="Q8:R8"/>
-    <mergeCell ref="S8:T8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="I9:K9"/>
-    <mergeCell ref="M9:N9"/>
-    <mergeCell ref="O9:P9"/>
-    <mergeCell ref="Q9:R9"/>
-    <mergeCell ref="S9:T9"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="M8:N8"/>
-    <mergeCell ref="B2:T2"/>
-    <mergeCell ref="B3:T3"/>
-    <mergeCell ref="B5:K5"/>
-    <mergeCell ref="M5:T5"/>
-    <mergeCell ref="B6:F7"/>
-    <mergeCell ref="G6:K7"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="O6:P6"/>
-    <mergeCell ref="Q6:R6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="O7:P7"/>
-    <mergeCell ref="Q7:R7"/>
-    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="B13:C17"/>
+    <mergeCell ref="D13:F17"/>
+    <mergeCell ref="G13:K13"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="I17:K17"/>
+    <mergeCell ref="M13:T13"/>
+    <mergeCell ref="N14:O14"/>
+    <mergeCell ref="I15:K16"/>
+    <mergeCell ref="N15:O15"/>
+    <mergeCell ref="N16:O16"/>
+    <mergeCell ref="I14:K14"/>
+    <mergeCell ref="N17:O17"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="G18:K18"/>
+    <mergeCell ref="N18:O18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="I19:K19"/>
+    <mergeCell ref="N19:O19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="I21:K21"/>
+    <mergeCell ref="B26:K27"/>
+    <mergeCell ref="C29:C30"/>
+    <mergeCell ref="H29:H30"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="G22:H24"/>
+    <mergeCell ref="I22:K24"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="D24:F24"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>

</xml_diff>